<commit_message>
Auto sync 2026-10-20 11:57:22
</commit_message>
<xml_diff>
--- a/outputs/logistics-review/最终职责-仓库只读导出.xlsx
+++ b/outputs/logistics-review/最终职责-仓库只读导出.xlsx
@@ -319,7 +319,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 11:56:35</t>
+          <t xml:space="preserve">2026-10-24 11:57:12</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -360,12 +360,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-22 07:56:35</t>
+          <t xml:space="preserve">2026-10-22 07:57:12</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 11:56:00</t>
+          <t xml:space="preserve">2026-10-20 11:57:00</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -388,12 +388,12 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 11:56:36</t>
+          <t xml:space="preserve">2026-10-20 11:57:12</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 11:56:36</t>
+          <t xml:space="preserve">2026-10-20 11:57:12</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19 11:56:35</t>
+          <t xml:space="preserve">2026-10-19 11:57:12</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -575,12 +575,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 11:56:35</t>
+          <t xml:space="preserve">2026-10-24 11:57:12</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 11:56:00</t>
+          <t xml:space="preserve">2026-10-20 11:57:00</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19 11:56:35</t>
+          <t xml:space="preserve">2026-10-19 11:57:12</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -650,12 +650,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 11:56:35</t>
+          <t xml:space="preserve">2026-10-24 11:57:12</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 11:56:00</t>
+          <t xml:space="preserve">2026-10-20 11:57:00</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">

</xml_diff>

<commit_message>
Auto sync 2026-10-20 13:12:24
</commit_message>
<xml_diff>
--- a/outputs/logistics-review/最终职责-仓库只读导出.xlsx
+++ b/outputs/logistics-review/最终职责-仓库只读导出.xlsx
@@ -319,7 +319,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 11:57:12</t>
+          <t xml:space="preserve">2026-10-24 13:12:12</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -360,12 +360,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-22 07:57:12</t>
+          <t xml:space="preserve">2026-10-22 09:12:12</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 11:57:00</t>
+          <t xml:space="preserve">2026-10-20 13:12:00</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -388,12 +388,12 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 11:57:12</t>
+          <t xml:space="preserve">2026-10-20 13:12:12</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 11:57:12</t>
+          <t xml:space="preserve">2026-10-20 13:12:12</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19 11:57:12</t>
+          <t xml:space="preserve">2026-10-19 13:12:12</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -575,12 +575,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 11:57:12</t>
+          <t xml:space="preserve">2026-10-24 13:12:12</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 11:57:00</t>
+          <t xml:space="preserve">2026-10-20 13:12:00</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19 11:57:12</t>
+          <t xml:space="preserve">2026-10-19 13:12:12</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -650,12 +650,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 11:57:12</t>
+          <t xml:space="preserve">2026-10-24 13:12:12</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 11:57:00</t>
+          <t xml:space="preserve">2026-10-20 13:12:00</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">

</xml_diff>

<commit_message>
Auto sync 2026-10-20 13:29:16
</commit_message>
<xml_diff>
--- a/outputs/logistics-review/最终职责-仓库只读导出.xlsx
+++ b/outputs/logistics-review/最终职责-仓库只读导出.xlsx
@@ -319,7 +319,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 13:12:12</t>
+          <t xml:space="preserve">2026-10-24 13:18:21</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -360,12 +360,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-22 09:12:12</t>
+          <t xml:space="preserve">2026-10-22 09:18:21</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:12:00</t>
+          <t xml:space="preserve">2026-10-20 13:18:00</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -388,12 +388,12 @@
       </c>
       <c r="AC2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:12:12</t>
+          <t xml:space="preserve">2026-10-20 13:18:22</t>
         </is>
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:12:12</t>
+          <t xml:space="preserve">2026-10-20 13:18:22</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19 13:12:12</t>
+          <t xml:space="preserve">2026-10-19 13:18:21</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -575,12 +575,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 13:12:12</t>
+          <t xml:space="preserve">2026-10-24 13:18:21</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:12:00</t>
+          <t xml:space="preserve">2026-10-20 13:18:00</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-19 13:12:12</t>
+          <t xml:space="preserve">2026-10-19 13:18:21</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -650,12 +650,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-24 13:12:12</t>
+          <t xml:space="preserve">2026-10-24 13:18:21</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-10-20 13:12:00</t>
+          <t xml:space="preserve">2026-10-20 13:18:00</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">

</xml_diff>